<commit_message>
save correct version of setup.xlsx
</commit_message>
<xml_diff>
--- a/WorkCampaign/ROVCleaver UniversalSetup.xlsx
+++ b/WorkCampaign/ROVCleaver UniversalSetup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/PythonProgs/ROVCleaver_on_Dropbox/WorkCampaign/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/TestInputFiles/TestCampaigns/Test GA Primary 1-2024/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F4CA90-6C99-DC4B-AB97-7214C36DB698}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0759BA38-6B68-2F46-85A5-22203A62A4AF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32320" yWindow="820" windowWidth="25940" windowHeight="14100" activeTab="3" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
+    <workbookView xWindow="3800" yWindow="2940" windowWidth="25940" windowHeight="14100" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="39" r:id="rId1"/>
@@ -518,7 +518,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1451" uniqueCount="724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="689">
   <si>
     <t>File</t>
   </si>
@@ -1558,9 +1558,6 @@
     <t>Pre Assigned</t>
   </si>
   <si>
-    <t>VA</t>
-  </si>
-  <si>
     <t>PDIID</t>
   </si>
   <si>
@@ -1639,55 +1636,19 @@
     <t>single files loaded - sample</t>
   </si>
   <si>
-    <t>General Election 7-2023</t>
-  </si>
-  <si>
-    <t>Carol 2023 HD65 - Fredericksburg.csv</t>
-  </si>
-  <si>
     <t>IDENTIFY DUPES</t>
   </si>
   <si>
     <t>PROCESS DUPLICATES</t>
   </si>
   <si>
-    <t>carol</t>
-  </si>
-  <si>
     <t>SuffolkCity</t>
   </si>
   <si>
-    <t>df.loc[df['dupe_id_field'].isin(['L','D','O']), 'remove'] = "Duplicate other than first"  # usually keep 'F', 'X' of choices: (F)irst, (L)ast, other (D)upe, (O)ther [not used], 'X':not dupe</t>
-  </si>
-  <si>
-    <t>df.loc[df['carol'] == True, 'remove'] = "Assigned to Carol"</t>
-  </si>
-  <si>
     <t>df['firstname'] +'#'+ df['lastname'] +'#'+ df['age'].astype(str) +'#'+ df['address'].str.replace('[ .,-]', '', regex=True)  +'#'+ df['city'].str.replace(r'[ .,-]', '', regex=True)</t>
   </si>
   <si>
     <t>pull_group</t>
-  </si>
-  <si>
-    <t>2023 HD29 - BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 HD58 - BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 HD73 - BIPOC.csv</t>
-  </si>
-  <si>
-    <t>pull_group, filename</t>
-  </si>
-  <si>
-    <t>Original by Carol</t>
-  </si>
-  <si>
-    <t>pulled 7/24/23</t>
-  </si>
-  <si>
-    <t>pull_group, remove</t>
   </si>
   <si>
     <t>**/Campaigns/VA General 7-2023/Output/</t>
@@ -1883,9 +1844,6 @@
     <t>Calhoun</t>
   </si>
   <si>
-    <t>county, pull_group</t>
-  </si>
-  <si>
     <t>ColonialHeightsCity</t>
   </si>
   <si>
@@ -2106,9 +2064,6 @@
   </si>
   <si>
     <t>False,("xl_str_pivot_field5","str"), ("xl_str_pivot_field5_by_cnt","bool"), ("xl_str_pivot_field5_all","bool")</t>
-  </si>
-  <si>
-    <t>VA General, Test duplicates, Non Deep South, Non-bilingual</t>
   </si>
   <si>
     <t>USEFUL IN NEW STATES/COUNTIES: whether to open a browser window for each concentrated address in report so you can research and enter a description and decide whether to remove. Most useful in new states/counties because prior should already be contained in cumulative "ROVCLEAVERAddressRemoveFile".  Often run on Combined file once Format files are created.  "Yes" allows ROVCleaver program to run with no intervention and open browser windows.  "Prompt by County" allows skipping counties that have been completed.  Set in conjunction with FileList FormatFile and ConcatFiles column choices.  Note: This may open a lot of browser windows first time through so you may want to check the concentrations and work on one or two counties at a time.</t>
@@ -2151,45 +2106,12 @@
     <t>custom_field</t>
   </si>
   <si>
-    <t>filename, custom_field</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>b</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>d</t>
-  </si>
-  <si>
-    <t>e</t>
-  </si>
-  <si>
-    <t>f</t>
-  </si>
-  <si>
-    <t>g</t>
-  </si>
-  <si>
-    <t>df['carol'] = df['pull_group'].map(lambda x: (True if x == 1 else False) )</t>
-  </si>
-  <si>
     <t># Use custom_field from filelist to set a variable</t>
   </si>
   <si>
     <t># Use 'pull_group' in filelist to identify CAROL group - Note that fields need to be added to 'Format File' list to be included on file</t>
   </si>
   <si>
-    <t>early_addresses</t>
-  </si>
-  <si>
-    <t>df['early_addresses'] = df['custom_field'].map(lambda x: (True if x in ['d','e'] else False) )</t>
-  </si>
-  <si>
     <t xml:space="preserve">Row 1 - Bold, no shading;  Column A - remove shading </t>
   </si>
   <si>
@@ -2197,51 +2119,6 @@
   </si>
   <si>
     <t>Columns C, D, E - notes unclesr; consider shifting columns further right</t>
-  </si>
-  <si>
-    <t>2023 HD20 BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 HD21 BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 HD22 - BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 HD72 - BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 HD84 BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 HD86 Black and Hispanic.csv</t>
-  </si>
-  <si>
-    <t>2023 HD97.csv</t>
-  </si>
-  <si>
-    <t>2023 SD16 BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 SD17 Black Voters All Counties.csv</t>
-  </si>
-  <si>
-    <t>2023 SD22 Black Hispanic.csv</t>
-  </si>
-  <si>
-    <t>2023 SD24 BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 SD25 BIPOC.csv</t>
-  </si>
-  <si>
-    <t>2023 SD27 Black and Hispanic.csv</t>
-  </si>
-  <si>
-    <t>Carol 2023 HD76 - Chesterfield.csv</t>
-  </si>
-  <si>
-    <t>pulled 7/7/23</t>
   </si>
   <si>
     <t>Columns B --&gt; G: Centered all data</t>
@@ -2311,9 +2188,6 @@
     <t>FILENAME OF CONCATENATED DATA (combined file)</t>
   </si>
   <si>
-    <t>Combined VA General 7-2023</t>
-  </si>
-  <si>
     <t>Don't need file extension (added by program). Best to include STATE in name</t>
   </si>
   <si>
@@ -2652,9 +2526,6 @@
     <t>Move to Key Data section?</t>
   </si>
   <si>
-    <t>&lt;&lt; non string data</t>
-  </si>
-  <si>
     <t>UNUSED ROWS BELOW</t>
   </si>
   <si>
@@ -2685,9 +2556,6 @@
     <t xml:space="preserve">  #  Use lagest number in pull_group on FileList?</t>
   </si>
   <si>
-    <t>Often blank, used if 'grouping'</t>
-  </si>
-  <si>
     <t>CAMPAIGN SPLIT VARIABLE(S)</t>
   </si>
   <si>
@@ -2703,27 +2571,12 @@
     <t>False,("xl_factory_vars","str",{'str_case':'l'})</t>
   </si>
   <si>
-    <t>age_group</t>
-  </si>
-  <si>
     <t># make up fields for testing</t>
   </si>
   <si>
-    <t>race</t>
-  </si>
-  <si>
-    <t>df['age_group'] = df['age'].map(lambda x: ('Young' if x &lt;50 else 'Senior') )</t>
-  </si>
-  <si>
-    <t>statecounty</t>
-  </si>
-  <si>
     <t>Almost always statecounty (used to separate files for Sincere along with factory_vars)</t>
   </si>
   <si>
-    <t>df['race'] = df['rownum'].map(lambda x: ('Hispanic' if x % 2==0 else 'Black') )</t>
-  </si>
-  <si>
     <t>False,("xl_campaign_vars","str",{'str_case':'l'})</t>
   </si>
   <si>
@@ -2733,9 +2586,6 @@
     <t>SORT OUTPUT:  group_vars +: 1 (testing) = zip, ADDRESS random WARNING;  2 = (testing) = zip, random WARNING; 3=RANDOM;  4/other  =  not sorted</t>
   </si>
   <si>
-    <t>race,  age_group</t>
-  </si>
-  <si>
     <t>remove using max_pull_group</t>
   </si>
   <si>
@@ -2752,6 +2602,51 @@
   </si>
   <si>
     <t># df.loc[df['filename'] == '2023 HD58 - BIPOC.csv', 'race'] = "Asian"</t>
+  </si>
+  <si>
+    <t>2024 GA Primary CD13 - BIPOC ver 2.csv</t>
+  </si>
+  <si>
+    <t>pulled 1/26/24. replaces files missing county.</t>
+  </si>
+  <si>
+    <t>2024 GA Primary CD6 - BIPOC ver 2.csv</t>
+  </si>
+  <si>
+    <t>GA Primary, CD 6 &amp; 13, BIPOC voters</t>
+  </si>
+  <si>
+    <t>GA</t>
+  </si>
+  <si>
+    <t>Combined GA Primary 1-2024</t>
+  </si>
+  <si>
+    <t>Primary 1-2024</t>
+  </si>
+  <si>
+    <t># df['race'] = df['rownum'].map(lambda x: ('Hispanic' if x % 2==0 else 'Black') )</t>
+  </si>
+  <si>
+    <t># df['age_group'] = df['age'].map(lambda x: ('Young' if x &lt;50 else 'Senior') )</t>
+  </si>
+  <si>
+    <t># df['carol'] = df['pull_group'].map(lambda x: (True if x == 1 else False) )</t>
+  </si>
+  <si>
+    <t># df['early_addresses'] = df['custom_field'].map(lambda x: (True if x in ['d','e'] else False) )</t>
+  </si>
+  <si>
+    <t>Often blank, used if 'grouping' with different scripts for each group</t>
+  </si>
+  <si>
+    <t>dupe_id_field</t>
+  </si>
+  <si>
+    <t>df.loc[df['dupe_id_field'].isin(['L','D','O']), 'remove'] = "Duplicate other than first"      # usually keep 'F', 'X' of choices: (F)irst, (L)ast, other (D)upe, (O)ther [not used], 'X':not dupe</t>
+  </si>
+  <si>
+    <t>&lt; any pull_groups not equal are flagged in remove</t>
   </si>
 </sst>
 </file>
@@ -3187,10 +3082,10 @@
     <border>
       <left/>
       <right/>
-      <top style="thick">
+      <top/>
+      <bottom style="thin">
         <color auto="1"/>
-      </top>
-      <bottom/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -3354,11 +3249,11 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="4" builtinId="3"/>
@@ -3682,14 +3577,14 @@
     <tabColor rgb="FFFFFF00"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AE194"/>
+  <dimension ref="A1:AD194"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="10" hidden="1" customWidth="1" outlineLevel="3"/>
     <col min="2" max="3" width="8.1640625" hidden="1" customWidth="1" outlineLevel="3"/>
     <col min="4" max="4" width="8.83203125" hidden="1" customWidth="1" outlineLevel="3"/>
     <col min="5" max="5" width="45" hidden="1" customWidth="1" outlineLevel="3"/>
-    <col min="6" max="6" width="38.6640625" style="79" hidden="1" customWidth="1" outlineLevel="2" collapsed="1"/>
+    <col min="6" max="6" width="38.6640625" style="79" hidden="1" customWidth="1" outlineLevel="2"/>
     <col min="7" max="7" width="59.1640625" customWidth="1" collapsed="1"/>
     <col min="8" max="8" width="14.6640625" customWidth="1"/>
     <col min="9" max="9" width="12.33203125" customWidth="1"/>
@@ -3699,28 +3594,28 @@
   <sheetData>
     <row r="1" spans="1:14" ht="24">
       <c r="A1" t="s">
-        <v>460</v>
+        <v>446</v>
       </c>
       <c r="B1" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="C1" t="s">
-        <v>461</v>
+        <v>447</v>
       </c>
       <c r="D1" t="s">
-        <v>466</v>
+        <v>452</v>
       </c>
       <c r="E1" t="s">
-        <v>462</v>
+        <v>448</v>
       </c>
       <c r="F1" s="79" t="s">
-        <v>482</v>
+        <v>468</v>
       </c>
       <c r="G1" s="64" t="s">
         <v>289</v>
       </c>
       <c r="J1" s="85" t="s">
-        <v>669</v>
+        <v>627</v>
       </c>
       <c r="K1" s="63"/>
       <c r="L1" s="63"/>
@@ -3743,7 +3638,7 @@
         <v>3</v>
       </c>
       <c r="G3" s="27" t="s">
-        <v>579</v>
+        <v>538</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="16" thickBot="1">
@@ -3754,10 +3649,10 @@
         <v>4</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>580</v>
+        <v>539</v>
       </c>
       <c r="L4" s="62" t="s">
-        <v>686</v>
+        <v>644</v>
       </c>
       <c r="M4" s="62"/>
       <c r="N4" s="14"/>
@@ -3776,19 +3671,19 @@
         <v>1</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>464</v>
+        <v>450</v>
       </c>
       <c r="F5" s="79" t="s">
-        <v>643</v>
+        <v>601</v>
       </c>
       <c r="G5" s="65" t="s">
-        <v>529</v>
+        <v>677</v>
       </c>
       <c r="H5" s="66" t="s">
-        <v>581</v>
+        <v>540</v>
       </c>
       <c r="L5" s="62" t="s">
-        <v>687</v>
+        <v>645</v>
       </c>
       <c r="M5" s="62"/>
       <c r="N5" s="14"/>
@@ -3801,7 +3696,7 @@
         <v>6</v>
       </c>
       <c r="M6" s="62" t="s">
-        <v>688</v>
+        <v>646</v>
       </c>
       <c r="N6" s="62"/>
     </row>
@@ -3813,7 +3708,7 @@
         <v>7</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>582</v>
+        <v>541</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="17" thickTop="1" thickBot="1">
@@ -3830,16 +3725,16 @@
         <v>1</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>465</v>
+        <v>451</v>
       </c>
       <c r="F8" s="79" t="s">
-        <v>644</v>
+        <v>602</v>
       </c>
       <c r="G8" s="65" t="s">
-        <v>346</v>
+        <v>678</v>
       </c>
       <c r="H8" s="66" t="s">
-        <v>583</v>
+        <v>542</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="16" thickTop="1">
@@ -3858,12 +3753,12 @@
         <v>10</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>584</v>
+        <v>543</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="17" thickTop="1" thickBot="1">
       <c r="A11" s="57" t="s">
-        <v>486</v>
+        <v>472</v>
       </c>
       <c r="B11">
         <v>62</v>
@@ -3875,16 +3770,16 @@
         <v>1</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>506</v>
+        <v>492</v>
       </c>
       <c r="F11" s="81" t="s">
-        <v>645</v>
+        <v>603</v>
       </c>
       <c r="G11" s="65" t="s">
-        <v>585</v>
+        <v>679</v>
       </c>
       <c r="H11" s="66" t="s">
-        <v>586</v>
+        <v>544</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="16" thickTop="1">
@@ -3904,12 +3799,12 @@
         <v>13</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>587</v>
+        <v>545</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="17" thickTop="1" thickBot="1">
       <c r="A14" s="57" t="s">
-        <v>487</v>
+        <v>473</v>
       </c>
       <c r="B14">
         <v>105</v>
@@ -3921,16 +3816,16 @@
         <v>1</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>507</v>
+        <v>493</v>
       </c>
       <c r="F14" s="79" t="s">
-        <v>646</v>
+        <v>604</v>
       </c>
       <c r="G14" s="65" t="s">
-        <v>373</v>
+        <v>680</v>
       </c>
       <c r="H14" s="66" t="s">
-        <v>588</v>
+        <v>546</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="16" thickTop="1">
@@ -3950,7 +3845,7 @@
         <v>16</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>702</v>
+        <v>658</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="17" thickTop="1" thickBot="1">
@@ -3967,16 +3862,16 @@
         <v>1</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>714</v>
+        <v>665</v>
       </c>
       <c r="F17" s="79" t="s">
-        <v>704</v>
+        <v>660</v>
       </c>
       <c r="G17" s="67" t="s">
-        <v>711</v>
+        <v>19</v>
       </c>
       <c r="H17" s="66" t="s">
-        <v>712</v>
+        <v>664</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="16" thickTop="1">
@@ -3996,7 +3891,7 @@
         <v>18.2</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>703</v>
+        <v>659</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="17" thickTop="1" thickBot="1">
@@ -4013,16 +3908,14 @@
         <v>1</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>706</v>
+        <v>662</v>
       </c>
       <c r="F20" s="79" t="s">
-        <v>705</v>
-      </c>
-      <c r="G20" s="67" t="s">
-        <v>717</v>
-      </c>
+        <v>661</v>
+      </c>
+      <c r="G20" s="67"/>
       <c r="H20" s="66" t="s">
-        <v>701</v>
+        <v>685</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="16" thickTop="1">
@@ -4030,7 +3923,7 @@
         <v>18.600000000000001</v>
       </c>
       <c r="G21" s="43" t="s">
-        <v>715</v>
+        <v>666</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="16" thickBot="1">
@@ -4041,7 +3934,7 @@
         <v>19</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>589</v>
+        <v>547</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="17" thickTop="1" thickBot="1">
@@ -4058,16 +3951,16 @@
         <v>1</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>470</v>
+        <v>456</v>
       </c>
       <c r="F23" s="81" t="s">
-        <v>647</v>
+        <v>605</v>
       </c>
       <c r="G23" s="67">
-        <v>1001</v>
+        <v>999999</v>
       </c>
       <c r="H23" s="68" t="s">
-        <v>590</v>
+        <v>548</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="16" thickTop="1">
@@ -4087,12 +3980,12 @@
         <v>22</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="17" thickTop="1" thickBot="1">
       <c r="A26" s="57" t="s">
-        <v>485</v>
+        <v>471</v>
       </c>
       <c r="B26">
         <v>35</v>
@@ -4104,13 +3997,13 @@
         <v>1</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>505</v>
+        <v>491</v>
       </c>
       <c r="G26" s="67" t="b">
         <v>1</v>
       </c>
       <c r="H26" s="66" t="s">
-        <v>591</v>
+        <v>549</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="16" thickTop="1">
@@ -4138,7 +4031,7 @@
         <v>26</v>
       </c>
       <c r="G29" s="27" t="s">
-        <v>592</v>
+        <v>550</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="19">
@@ -4149,7 +4042,7 @@
         <v>27</v>
       </c>
       <c r="G30" s="69" t="s">
-        <v>593</v>
+        <v>551</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -4160,21 +4053,21 @@
         <v>28</v>
       </c>
       <c r="F31" s="79" t="s">
-        <v>649</v>
+        <v>607</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>594</v>
+        <v>552</v>
       </c>
       <c r="H31" s="86" t="s">
-        <v>670</v>
+        <v>628</v>
       </c>
       <c r="L31" s="62" t="s">
-        <v>689</v>
+        <v>647</v>
       </c>
       <c r="M31" s="62"/>
       <c r="N31" s="14"/>
     </row>
-    <row r="32" spans="1:14" ht="16" thickBot="1">
+    <row r="32" spans="1:14">
       <c r="B32">
         <v>14</v>
       </c>
@@ -4182,10 +4075,10 @@
         <v>29</v>
       </c>
       <c r="G32" s="66" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="33" spans="1:31" ht="16" thickTop="1">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23">
       <c r="A33" t="b">
         <v>1</v>
       </c>
@@ -4199,13 +4092,13 @@
         <v>1</v>
       </c>
       <c r="E33" s="90" t="s">
-        <v>467</v>
+        <v>453</v>
       </c>
       <c r="F33" s="91" t="s">
-        <v>532</v>
+        <v>517</v>
       </c>
       <c r="G33" s="95" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="H33" s="95" t="s">
         <v>201</v>
@@ -4234,25 +4127,14 @@
       <c r="P33" s="95" t="s">
         <v>210</v>
       </c>
-      <c r="Q33" s="96" t="s">
+      <c r="Q33" s="60" t="s">
         <v>211</v>
       </c>
-      <c r="R33" s="96"/>
-      <c r="S33" s="96"/>
-      <c r="T33" s="96"/>
-      <c r="U33" s="96"/>
-      <c r="V33" s="96"/>
-      <c r="W33" s="96"/>
-      <c r="X33" s="96"/>
-      <c r="Y33" s="96"/>
-      <c r="Z33" s="96"/>
-      <c r="AA33" s="96"/>
-      <c r="AB33" s="96"/>
-      <c r="AC33" s="96"/>
-      <c r="AD33" s="96"/>
-      <c r="AE33" s="96"/>
-    </row>
-    <row r="34" spans="1:31" ht="16" thickBot="1">
+      <c r="R33" s="60"/>
+      <c r="S33" s="60"/>
+      <c r="T33" s="60"/>
+    </row>
+    <row r="34" spans="1:23">
       <c r="A34" t="b">
         <v>1</v>
       </c>
@@ -4266,13 +4148,13 @@
         <v>1</v>
       </c>
       <c r="E34" s="90" t="s">
-        <v>468</v>
+        <v>454</v>
       </c>
       <c r="F34" s="93" t="s">
         <v>277</v>
       </c>
       <c r="G34" s="89" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="H34" s="89" t="s">
         <v>20</v>
@@ -4307,29 +4189,10 @@
       <c r="R34" s="89" t="s">
         <v>14</v>
       </c>
-      <c r="S34" s="89" t="s">
-        <v>377</v>
-      </c>
-      <c r="T34" s="92" t="s">
-        <v>554</v>
-      </c>
-      <c r="U34" s="89" t="s">
-        <v>709</v>
-      </c>
-      <c r="V34" s="89" t="s">
-        <v>707</v>
-      </c>
-      <c r="W34" s="89"/>
-      <c r="X34" s="89"/>
-      <c r="Y34" s="89"/>
-      <c r="Z34" s="89"/>
-      <c r="AA34" s="89"/>
-      <c r="AB34" s="89"/>
-      <c r="AC34" s="89"/>
-      <c r="AD34" s="89"/>
-      <c r="AE34" s="89"/>
-    </row>
-    <row r="35" spans="1:31" ht="17" thickTop="1" thickBot="1">
+      <c r="S34" s="89"/>
+      <c r="T34" s="92"/>
+    </row>
+    <row r="35" spans="1:23">
       <c r="A35" t="b">
         <v>1</v>
       </c>
@@ -4343,42 +4206,29 @@
         <v>1</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>469</v>
+        <v>455</v>
       </c>
       <c r="F35" s="81" t="s">
-        <v>648</v>
-      </c>
-      <c r="G35" s="97"/>
-      <c r="H35" s="98"/>
-      <c r="I35" s="98"/>
-      <c r="J35" s="99" t="s">
+        <v>606</v>
+      </c>
+      <c r="G35" s="96"/>
+      <c r="H35" s="97"/>
+      <c r="I35" s="97"/>
+      <c r="J35" s="98" t="s">
         <v>270</v>
       </c>
-      <c r="K35" s="94" t="s">
-        <v>690</v>
-      </c>
-      <c r="L35" s="94"/>
-      <c r="M35" s="94"/>
-      <c r="N35" s="94"/>
-      <c r="O35" s="94"/>
-      <c r="P35" s="94"/>
-      <c r="Q35" s="94"/>
-      <c r="R35" s="94"/>
-      <c r="S35" s="94"/>
-      <c r="T35" s="94"/>
-      <c r="U35" s="94"/>
-      <c r="V35" s="94"/>
-      <c r="W35" s="94"/>
-      <c r="X35" s="94"/>
-      <c r="Y35" s="94"/>
-      <c r="Z35" s="94"/>
-      <c r="AA35" s="94"/>
-      <c r="AB35" s="94"/>
-      <c r="AC35" s="94"/>
-      <c r="AD35" s="94"/>
-      <c r="AE35" s="94"/>
-    </row>
-    <row r="36" spans="1:31" ht="16" thickTop="1">
+      <c r="K35" s="99"/>
+      <c r="L35" s="99"/>
+      <c r="M35" s="99"/>
+      <c r="N35" s="99"/>
+      <c r="O35" s="99"/>
+      <c r="P35" s="99"/>
+      <c r="Q35" s="99"/>
+      <c r="R35" s="99"/>
+      <c r="S35" s="99"/>
+      <c r="T35" s="99"/>
+    </row>
+    <row r="36" spans="1:23">
       <c r="B36">
         <v>149</v>
       </c>
@@ -4386,7 +4236,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:31" ht="16" thickBot="1">
+    <row r="37" spans="1:23" ht="16" thickBot="1">
       <c r="B37">
         <v>150</v>
       </c>
@@ -4394,15 +4244,15 @@
         <v>34</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>596</v>
+        <v>554</v>
       </c>
       <c r="H37" s="66" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="38" spans="1:31" ht="17" thickTop="1" thickBot="1">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" ht="17" thickTop="1" thickBot="1">
       <c r="A38" s="57" t="s">
-        <v>489</v>
+        <v>475</v>
       </c>
       <c r="B38">
         <v>151</v>
@@ -4414,10 +4264,10 @@
         <v>1</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>518</v>
+        <v>504</v>
       </c>
       <c r="F38" s="79" t="s">
-        <v>664</v>
+        <v>622</v>
       </c>
       <c r="G38" s="94" t="s">
         <v>54</v>
@@ -4433,7 +4283,7 @@
       <c r="P38" s="94"/>
       <c r="Q38" s="94"/>
     </row>
-    <row r="39" spans="1:31" ht="16" thickTop="1">
+    <row r="39" spans="1:23" ht="16" thickTop="1">
       <c r="B39">
         <v>152</v>
       </c>
@@ -4441,7 +4291,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="40" spans="1:31" ht="16" thickBot="1">
+    <row r="40" spans="1:23" ht="16" thickBot="1">
       <c r="B40">
         <v>155</v>
       </c>
@@ -4449,13 +4299,13 @@
         <v>37</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>598</v>
+        <v>556</v>
       </c>
       <c r="H40" s="66" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="41" spans="1:31" ht="17" thickTop="1" thickBot="1">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" ht="17" thickTop="1" thickBot="1">
       <c r="A41" t="b">
         <v>1</v>
       </c>
@@ -4469,10 +4319,10 @@
         <v>1</v>
       </c>
       <c r="E41" s="15" t="s">
-        <v>472</v>
+        <v>458</v>
       </c>
       <c r="F41" s="79" t="s">
-        <v>665</v>
+        <v>623</v>
       </c>
       <c r="G41" s="94" t="s">
         <v>20</v>
@@ -4502,11 +4352,9 @@
         <v>19</v>
       </c>
       <c r="P41" s="94" t="s">
-        <v>363</v>
-      </c>
-      <c r="Q41" s="94" t="s">
-        <v>382</v>
-      </c>
+        <v>362</v>
+      </c>
+      <c r="Q41" s="94"/>
       <c r="R41" s="94"/>
       <c r="S41" s="94"/>
       <c r="T41" s="94"/>
@@ -4514,7 +4362,7 @@
       <c r="V41" s="94"/>
       <c r="W41" s="94"/>
     </row>
-    <row r="42" spans="1:31" ht="16" thickTop="1">
+    <row r="42" spans="1:23" ht="16" thickTop="1">
       <c r="B42">
         <v>157</v>
       </c>
@@ -4523,7 +4371,7 @@
       </c>
       <c r="F42" s="81"/>
     </row>
-    <row r="43" spans="1:31" ht="16" thickBot="1">
+    <row r="43" spans="1:23" ht="16" thickBot="1">
       <c r="B43">
         <v>191</v>
       </c>
@@ -4531,12 +4379,12 @@
         <v>40</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="44" spans="1:31" ht="17" thickTop="1" thickBot="1">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" ht="17" thickTop="1" thickBot="1">
       <c r="A44" s="57" t="s">
-        <v>491</v>
+        <v>477</v>
       </c>
       <c r="B44">
         <v>192</v>
@@ -4548,19 +4396,19 @@
         <v>1</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>509</v>
+        <v>495</v>
       </c>
       <c r="F44" s="79" t="s">
         <v>279</v>
       </c>
       <c r="G44" s="71" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="H44" s="66" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="45" spans="1:31" ht="16" thickTop="1">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" ht="16" thickTop="1">
       <c r="B45">
         <v>193</v>
       </c>
@@ -4568,7 +4416,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:31" ht="16" thickBot="1">
+    <row r="46" spans="1:23" ht="16" thickBot="1">
       <c r="B46">
         <v>194</v>
       </c>
@@ -4576,13 +4424,13 @@
         <v>43</v>
       </c>
       <c r="G46" t="s">
-        <v>602</v>
+        <v>560</v>
       </c>
       <c r="H46" s="66"/>
     </row>
-    <row r="47" spans="1:31" ht="17" thickTop="1" thickBot="1">
+    <row r="47" spans="1:23" ht="17" thickTop="1" thickBot="1">
       <c r="A47" s="57" t="s">
-        <v>492</v>
+        <v>478</v>
       </c>
       <c r="B47">
         <v>195</v>
@@ -4594,7 +4442,7 @@
         <v>1</v>
       </c>
       <c r="E47" s="15" t="s">
-        <v>510</v>
+        <v>496</v>
       </c>
       <c r="F47" s="79" t="s">
         <v>278</v>
@@ -4603,7 +4451,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="48" spans="1:31" ht="16" thickTop="1">
+    <row r="48" spans="1:23" ht="16" thickTop="1">
       <c r="B48">
         <v>196</v>
       </c>
@@ -4624,7 +4472,7 @@
     </row>
     <row r="50" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A50" s="57" t="s">
-        <v>490</v>
+        <v>476</v>
       </c>
       <c r="B50">
         <v>188</v>
@@ -4636,16 +4484,16 @@
         <v>1</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>508</v>
+        <v>494</v>
       </c>
       <c r="F50" s="79" t="s">
-        <v>650</v>
+        <v>608</v>
       </c>
       <c r="G50" s="72" t="b">
         <v>0</v>
       </c>
       <c r="H50" s="66" t="s">
-        <v>651</v>
+        <v>609</v>
       </c>
     </row>
     <row r="51" spans="1:16" ht="16" thickTop="1">
@@ -4664,10 +4512,10 @@
         <v>49</v>
       </c>
       <c r="G52" s="69" t="s">
-        <v>603</v>
+        <v>561</v>
       </c>
       <c r="H52" s="66" t="s">
-        <v>604</v>
+        <v>562</v>
       </c>
     </row>
     <row r="53" spans="1:16" ht="49" thickBot="1">
@@ -4678,13 +4526,13 @@
         <v>50</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>605</v>
+        <v>563</v>
       </c>
       <c r="H53" s="35" t="s">
-        <v>606</v>
+        <v>564</v>
       </c>
       <c r="I53" s="35" t="s">
-        <v>607</v>
+        <v>565</v>
       </c>
     </row>
     <row r="54" spans="1:16" ht="17" thickTop="1" thickBot="1">
@@ -4701,13 +4549,13 @@
         <v>1</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>524</v>
+        <v>510</v>
       </c>
       <c r="F54" s="79" t="s">
-        <v>534</v>
+        <v>519</v>
       </c>
       <c r="G54" s="71" t="s">
-        <v>386</v>
+        <v>686</v>
       </c>
       <c r="H54" s="73" t="b">
         <v>0</v>
@@ -4730,7 +4578,7 @@
         <v>1</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>525</v>
+        <v>511</v>
       </c>
       <c r="F55" s="81"/>
       <c r="G55" s="71"/>
@@ -4755,11 +4603,9 @@
         <v>1</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>526</v>
-      </c>
-      <c r="G56" s="71" t="s">
-        <v>454</v>
-      </c>
+        <v>512</v>
+      </c>
+      <c r="G56" s="71"/>
       <c r="H56" s="71" t="b">
         <v>0</v>
       </c>
@@ -4781,11 +4627,9 @@
         <v>1</v>
       </c>
       <c r="E57" s="15" t="s">
-        <v>527</v>
-      </c>
-      <c r="G57" s="71" t="s">
-        <v>389</v>
-      </c>
+        <v>513</v>
+      </c>
+      <c r="G57" s="71"/>
       <c r="H57" s="71" t="b">
         <v>1</v>
       </c>
@@ -4807,11 +4651,9 @@
         <v>1</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>528</v>
-      </c>
-      <c r="G58" s="71" t="s">
-        <v>543</v>
-      </c>
+        <v>514</v>
+      </c>
+      <c r="G58" s="71"/>
       <c r="H58" s="71" t="b">
         <v>0</v>
       </c>
@@ -4844,7 +4686,7 @@
         <v>58</v>
       </c>
       <c r="G61" s="69" t="s">
-        <v>609</v>
+        <v>567</v>
       </c>
     </row>
     <row r="62" spans="1:16" ht="16" thickBot="1">
@@ -4855,10 +4697,10 @@
         <v>59</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>608</v>
+        <v>566</v>
       </c>
       <c r="L62" s="62" t="s">
-        <v>654</v>
+        <v>612</v>
       </c>
       <c r="M62" s="61"/>
       <c r="N62" s="61"/>
@@ -4879,16 +4721,16 @@
         <v>1</v>
       </c>
       <c r="E63" t="s">
-        <v>471</v>
+        <v>457</v>
       </c>
       <c r="F63" s="79" t="s">
-        <v>653</v>
+        <v>611</v>
       </c>
       <c r="G63" s="71" t="s">
         <v>276</v>
       </c>
       <c r="H63" s="66" t="s">
-        <v>652</v>
+        <v>610</v>
       </c>
     </row>
     <row r="64" spans="1:16" ht="16" thickTop="1">
@@ -4907,12 +4749,12 @@
         <v>62</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>610</v>
+        <v>568</v>
       </c>
     </row>
     <row r="66" spans="1:15" ht="17" thickTop="1" thickBot="1">
       <c r="A66" s="57" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="B66">
         <v>24</v>
@@ -4924,16 +4766,16 @@
         <v>1</v>
       </c>
       <c r="E66" s="15" t="s">
-        <v>504</v>
+        <v>490</v>
       </c>
       <c r="F66" s="79" t="s">
-        <v>530</v>
+        <v>515</v>
       </c>
       <c r="G66" s="72">
         <v>3</v>
       </c>
       <c r="H66" s="66" t="s">
-        <v>611</v>
+        <v>569</v>
       </c>
     </row>
     <row r="67" spans="1:15" ht="16" thickTop="1">
@@ -4952,13 +4794,13 @@
         <v>65</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>656</v>
+        <v>614</v>
       </c>
       <c r="H68" s="66" t="s">
-        <v>657</v>
+        <v>615</v>
       </c>
       <c r="L68" s="62" t="s">
-        <v>612</v>
+        <v>570</v>
       </c>
       <c r="M68" s="61"/>
       <c r="N68" s="61"/>
@@ -4978,13 +4820,13 @@
         <v>1</v>
       </c>
       <c r="E69" s="15" t="s">
-        <v>535</v>
+        <v>520</v>
       </c>
       <c r="F69" s="79" t="s">
-        <v>655</v>
+        <v>613</v>
       </c>
       <c r="G69" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
     </row>
     <row r="70" spans="1:15">
@@ -5003,16 +4845,16 @@
         <v>68</v>
       </c>
       <c r="G71" s="32" t="s">
-        <v>658</v>
+        <v>616</v>
       </c>
       <c r="H71" s="82" t="s">
-        <v>659</v>
+        <v>617</v>
       </c>
       <c r="I71" s="14"/>
       <c r="J71" s="78"/>
       <c r="K71" s="78"/>
       <c r="L71" s="62" t="s">
-        <v>667</v>
+        <v>625</v>
       </c>
       <c r="M71" s="61"/>
       <c r="N71" s="61"/>
@@ -5032,16 +4874,16 @@
         <v>1</v>
       </c>
       <c r="E72" s="15" t="s">
-        <v>480</v>
+        <v>466</v>
       </c>
       <c r="F72" s="79" t="s">
-        <v>541</v>
+        <v>526</v>
       </c>
       <c r="G72" s="71" t="s">
-        <v>481</v>
+        <v>467</v>
       </c>
       <c r="L72" s="62" t="s">
-        <v>612</v>
+        <v>570</v>
       </c>
       <c r="M72" s="61"/>
       <c r="N72" s="61"/>
@@ -5063,12 +4905,12 @@
         <v>71</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>613</v>
+        <v>571</v>
       </c>
     </row>
     <row r="75" spans="1:15" ht="17" thickTop="1" thickBot="1">
       <c r="A75" s="57" t="s">
-        <v>493</v>
+        <v>479</v>
       </c>
       <c r="B75">
         <v>200</v>
@@ -5080,16 +4922,16 @@
         <v>1</v>
       </c>
       <c r="E75" s="15" t="s">
-        <v>511</v>
+        <v>497</v>
       </c>
       <c r="F75" s="79" t="s">
-        <v>666</v>
+        <v>624</v>
       </c>
       <c r="G75" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H75" s="66" t="s">
-        <v>614</v>
+        <v>572</v>
       </c>
     </row>
     <row r="76" spans="1:15" ht="16" thickTop="1">
@@ -5108,17 +4950,17 @@
         <v>74</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>615</v>
+        <v>573</v>
       </c>
       <c r="L77" s="62" t="s">
-        <v>616</v>
+        <v>574</v>
       </c>
       <c r="M77" s="62"/>
       <c r="N77" s="14"/>
     </row>
     <row r="78" spans="1:15" ht="17" thickTop="1" thickBot="1">
       <c r="A78" s="57" t="s">
-        <v>494</v>
+        <v>480</v>
       </c>
       <c r="B78">
         <v>211</v>
@@ -5130,16 +4972,16 @@
         <v>1</v>
       </c>
       <c r="E78" s="15" t="s">
-        <v>512</v>
+        <v>498</v>
       </c>
       <c r="F78" s="83" t="s">
-        <v>533</v>
+        <v>518</v>
       </c>
       <c r="G78" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H78" s="66" t="s">
-        <v>617</v>
+        <v>575</v>
       </c>
     </row>
     <row r="79" spans="1:15" ht="16" thickTop="1">
@@ -5158,12 +5000,12 @@
         <v>77</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>618</v>
+        <v>576</v>
       </c>
     </row>
     <row r="81" spans="1:30" ht="17" thickTop="1" thickBot="1">
       <c r="A81" t="s">
-        <v>495</v>
+        <v>481</v>
       </c>
       <c r="B81">
         <v>215</v>
@@ -5175,16 +5017,16 @@
         <v>1</v>
       </c>
       <c r="E81" s="15" t="s">
-        <v>520</v>
+        <v>506</v>
       </c>
       <c r="F81" s="79" t="s">
-        <v>660</v>
+        <v>618</v>
       </c>
       <c r="G81" s="72" t="s">
         <v>196</v>
       </c>
       <c r="H81" s="66" t="s">
-        <v>619</v>
+        <v>577</v>
       </c>
     </row>
     <row r="82" spans="1:30" ht="16" thickTop="1">
@@ -5211,7 +5053,7 @@
         <v>81</v>
       </c>
       <c r="G84" s="69" t="s">
-        <v>620</v>
+        <v>578</v>
       </c>
     </row>
     <row r="85" spans="1:30" ht="16" thickBot="1">
@@ -5222,12 +5064,12 @@
         <v>82</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>621</v>
+        <v>579</v>
       </c>
     </row>
     <row r="86" spans="1:30" ht="17" thickTop="1" thickBot="1">
       <c r="A86" s="57" t="s">
-        <v>498</v>
+        <v>484</v>
       </c>
       <c r="B86">
         <v>248</v>
@@ -5239,16 +5081,16 @@
         <v>1</v>
       </c>
       <c r="E86" s="15" t="s">
-        <v>513</v>
+        <v>499</v>
       </c>
       <c r="F86" s="79" t="s">
-        <v>661</v>
+        <v>619</v>
       </c>
       <c r="G86" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H86" s="66" t="s">
-        <v>622</v>
+        <v>580</v>
       </c>
     </row>
     <row r="87" spans="1:30" ht="16" thickTop="1">
@@ -5268,12 +5110,12 @@
         <v>85</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>623</v>
+        <v>581</v>
       </c>
     </row>
     <row r="89" spans="1:30" ht="17" thickTop="1" thickBot="1">
       <c r="A89" s="57" t="s">
-        <v>499</v>
+        <v>485</v>
       </c>
       <c r="B89">
         <v>253</v>
@@ -5285,16 +5127,16 @@
         <v>1</v>
       </c>
       <c r="E89" s="15" t="s">
-        <v>514</v>
+        <v>500</v>
       </c>
       <c r="F89" s="79" t="s">
-        <v>662</v>
+        <v>620</v>
       </c>
       <c r="G89" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H89" s="66" t="s">
-        <v>624</v>
+        <v>582</v>
       </c>
     </row>
     <row r="90" spans="1:30" ht="16" thickTop="1">
@@ -5313,10 +5155,10 @@
         <v>88</v>
       </c>
       <c r="G91" s="84" t="s">
-        <v>716</v>
+        <v>667</v>
       </c>
       <c r="N91" s="62" t="s">
-        <v>625</v>
+        <v>583</v>
       </c>
       <c r="O91" s="61"/>
       <c r="P91" s="61"/>
@@ -5325,7 +5167,7 @@
     </row>
     <row r="92" spans="1:30" ht="17" thickTop="1" thickBot="1">
       <c r="A92" s="57" t="s">
-        <v>484</v>
+        <v>470</v>
       </c>
       <c r="B92">
         <v>29</v>
@@ -5337,16 +5179,16 @@
         <v>1</v>
       </c>
       <c r="E92" s="15" t="s">
+        <v>502</v>
+      </c>
+      <c r="F92" s="83" t="s">
         <v>516</v>
       </c>
-      <c r="F92" s="83" t="s">
-        <v>531</v>
-      </c>
       <c r="G92" s="74">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H92" s="66" t="s">
-        <v>626</v>
+        <v>584</v>
       </c>
     </row>
     <row r="93" spans="1:30" ht="16" thickTop="1">
@@ -5360,7 +5202,7 @@
         <v>266</v>
       </c>
       <c r="L93" s="62" t="s">
-        <v>627</v>
+        <v>585</v>
       </c>
       <c r="M93" s="61"/>
       <c r="N93" s="61"/>
@@ -5381,13 +5223,13 @@
         <v>92</v>
       </c>
       <c r="G95" s="1" t="s">
-        <v>628</v>
+        <v>586</v>
       </c>
       <c r="I95" s="17"/>
     </row>
     <row r="96" spans="1:30" ht="17" thickTop="1" thickBot="1">
       <c r="A96" s="57" t="s">
-        <v>488</v>
+        <v>474</v>
       </c>
       <c r="B96">
         <v>110</v>
@@ -5399,16 +5241,16 @@
         <v>1</v>
       </c>
       <c r="E96" s="15" t="s">
-        <v>517</v>
+        <v>503</v>
       </c>
       <c r="F96" s="79" t="s">
-        <v>668</v>
+        <v>626</v>
       </c>
       <c r="G96" s="74">
         <v>25000</v>
       </c>
       <c r="H96" s="66" t="s">
-        <v>629</v>
+        <v>587</v>
       </c>
       <c r="J96" s="75"/>
       <c r="K96" s="75"/>
@@ -5437,7 +5279,7 @@
         <v>96</v>
       </c>
       <c r="G99" s="27" t="s">
-        <v>639</v>
+        <v>597</v>
       </c>
     </row>
     <row r="100" spans="1:16" ht="16" thickBot="1">
@@ -5448,16 +5290,16 @@
         <v>97</v>
       </c>
       <c r="G100" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="H100" s="87" t="s">
         <v>630</v>
-      </c>
-      <c r="H100" s="87" t="s">
-        <v>672</v>
       </c>
       <c r="I100" s="78"/>
     </row>
     <row r="101" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A101" t="s">
-        <v>473</v>
+        <v>459</v>
       </c>
       <c r="B101">
         <v>220</v>
@@ -5469,19 +5311,19 @@
         <v>1</v>
       </c>
       <c r="E101" s="15" t="s">
-        <v>474</v>
+        <v>460</v>
       </c>
       <c r="F101" s="79" t="s">
-        <v>671</v>
+        <v>629</v>
       </c>
       <c r="G101" s="72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H101" s="66" t="s">
-        <v>591</v>
+        <v>549</v>
       </c>
       <c r="L101" s="62" t="s">
-        <v>640</v>
+        <v>598</v>
       </c>
       <c r="M101" s="62"/>
       <c r="N101" s="62"/>
@@ -5503,15 +5345,15 @@
         <v>100</v>
       </c>
       <c r="G103" s="1" t="s">
-        <v>631</v>
+        <v>589</v>
       </c>
       <c r="H103" s="66" t="s">
-        <v>632</v>
+        <v>590</v>
       </c>
     </row>
     <row r="104" spans="1:16" s="79" customFormat="1" ht="17" thickTop="1" thickBot="1">
       <c r="A104" s="79" t="s">
-        <v>479</v>
+        <v>465</v>
       </c>
       <c r="B104" s="79">
         <v>224</v>
@@ -5523,19 +5365,19 @@
         <v>1</v>
       </c>
       <c r="E104" s="81" t="s">
-        <v>521</v>
+        <v>507</v>
       </c>
       <c r="F104" s="88" t="s">
-        <v>673</v>
+        <v>631</v>
       </c>
       <c r="G104" s="71" t="s">
         <v>284</v>
       </c>
       <c r="H104" s="66" t="s">
-        <v>633</v>
+        <v>591</v>
       </c>
       <c r="L104" s="62" t="s">
-        <v>685</v>
+        <v>643</v>
       </c>
       <c r="M104" s="62"/>
       <c r="N104" s="62"/>
@@ -5558,15 +5400,15 @@
         <v>103</v>
       </c>
       <c r="G106" s="1" t="s">
-        <v>634</v>
+        <v>592</v>
       </c>
       <c r="H106" s="66" t="s">
-        <v>675</v>
+        <v>633</v>
       </c>
     </row>
     <row r="107" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A107" t="s">
-        <v>476</v>
+        <v>462</v>
       </c>
       <c r="B107">
         <v>229</v>
@@ -5578,16 +5420,16 @@
         <v>1</v>
       </c>
       <c r="E107" s="15" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="F107" s="88" t="s">
-        <v>674</v>
+        <v>632</v>
       </c>
       <c r="G107" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H107" s="66" t="s">
-        <v>635</v>
+        <v>593</v>
       </c>
     </row>
     <row r="108" spans="1:16" ht="16" thickTop="1">
@@ -5606,12 +5448,12 @@
         <v>106</v>
       </c>
       <c r="G109" s="1" t="s">
-        <v>636</v>
+        <v>594</v>
       </c>
     </row>
     <row r="110" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A110" s="57" t="s">
-        <v>496</v>
+        <v>482</v>
       </c>
       <c r="B110">
         <v>233</v>
@@ -5623,19 +5465,19 @@
         <v>1</v>
       </c>
       <c r="E110" s="15" t="s">
-        <v>522</v>
+        <v>508</v>
       </c>
       <c r="F110" s="88" t="s">
-        <v>681</v>
+        <v>639</v>
       </c>
       <c r="G110" s="71" t="s">
         <v>285</v>
       </c>
       <c r="H110" s="66" t="s">
-        <v>633</v>
+        <v>591</v>
       </c>
       <c r="L110" s="62" t="s">
-        <v>676</v>
+        <v>634</v>
       </c>
       <c r="M110" s="62"/>
       <c r="N110" s="62"/>
@@ -5658,15 +5500,15 @@
         <v>109</v>
       </c>
       <c r="G112" s="1" t="s">
-        <v>637</v>
+        <v>595</v>
       </c>
       <c r="H112" s="66" t="s">
-        <v>677</v>
+        <v>635</v>
       </c>
     </row>
     <row r="113" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A113" t="s">
-        <v>477</v>
+        <v>463</v>
       </c>
       <c r="B113">
         <v>238</v>
@@ -5678,16 +5520,16 @@
         <v>1</v>
       </c>
       <c r="E113" s="15" t="s">
-        <v>478</v>
+        <v>464</v>
       </c>
       <c r="F113" s="88" t="s">
-        <v>678</v>
+        <v>636</v>
       </c>
       <c r="G113" s="72" t="b">
         <v>1</v>
       </c>
       <c r="H113" s="66" t="s">
-        <v>635</v>
+        <v>593</v>
       </c>
     </row>
     <row r="114" spans="1:16" ht="16" thickTop="1">
@@ -5706,12 +5548,12 @@
         <v>112</v>
       </c>
       <c r="G115" s="1" t="s">
-        <v>638</v>
+        <v>596</v>
       </c>
     </row>
     <row r="116" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A116" s="57" t="s">
-        <v>497</v>
+        <v>483</v>
       </c>
       <c r="B116">
         <v>242</v>
@@ -5723,19 +5565,19 @@
         <v>1</v>
       </c>
       <c r="E116" s="15" t="s">
-        <v>523</v>
+        <v>509</v>
       </c>
       <c r="F116" s="88" t="s">
-        <v>679</v>
+        <v>637</v>
       </c>
       <c r="G116" s="71" t="s">
         <v>286</v>
       </c>
       <c r="H116" s="66" t="s">
-        <v>633</v>
+        <v>591</v>
       </c>
       <c r="L116" s="62" t="s">
-        <v>680</v>
+        <v>638</v>
       </c>
       <c r="M116" s="62"/>
       <c r="N116" s="62"/>
@@ -5777,12 +5619,12 @@
         <v>117</v>
       </c>
       <c r="G120" t="s">
-        <v>682</v>
+        <v>640</v>
       </c>
     </row>
     <row r="121" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A121" s="57" t="s">
-        <v>500</v>
+        <v>486</v>
       </c>
       <c r="B121">
         <v>289</v>
@@ -5794,16 +5636,16 @@
         <v>1</v>
       </c>
       <c r="E121" s="15" t="s">
-        <v>515</v>
+        <v>501</v>
       </c>
       <c r="F121" s="88" t="s">
-        <v>684</v>
+        <v>642</v>
       </c>
       <c r="G121" s="72" t="b">
         <v>0</v>
       </c>
       <c r="H121" s="66" t="s">
-        <v>683</v>
+        <v>641</v>
       </c>
     </row>
     <row r="122" spans="1:16" ht="16" thickTop="1">
@@ -5828,7 +5670,7 @@
     </row>
     <row r="124" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A124" s="57" t="s">
-        <v>501</v>
+        <v>487</v>
       </c>
       <c r="B124">
         <v>294</v>
@@ -5840,10 +5682,10 @@
         <v>1</v>
       </c>
       <c r="E124" s="15" t="s">
-        <v>536</v>
+        <v>521</v>
       </c>
       <c r="F124" s="83" t="s">
-        <v>538</v>
+        <v>523</v>
       </c>
       <c r="G124" s="70" t="s">
         <v>193</v>
@@ -5865,17 +5707,17 @@
         <v>123</v>
       </c>
       <c r="G126" s="84" t="s">
-        <v>663</v>
+        <v>621</v>
       </c>
       <c r="N126" s="76" t="s">
-        <v>641</v>
+        <v>599</v>
       </c>
       <c r="O126" s="61"/>
       <c r="P126" s="61"/>
     </row>
     <row r="127" spans="1:16" ht="17" thickTop="1" thickBot="1">
       <c r="A127" s="57" t="s">
-        <v>502</v>
+        <v>488</v>
       </c>
       <c r="B127">
         <v>299</v>
@@ -5887,10 +5729,10 @@
         <v>1</v>
       </c>
       <c r="E127" s="15" t="s">
-        <v>537</v>
+        <v>522</v>
       </c>
       <c r="F127" s="83" t="s">
-        <v>539</v>
+        <v>524</v>
       </c>
       <c r="G127" s="70" t="s">
         <v>191</v>
@@ -5922,12 +5764,12 @@
       <c r="K129" s="9"/>
       <c r="L129" s="9"/>
       <c r="N129" s="62" t="s">
-        <v>642</v>
+        <v>600</v>
       </c>
     </row>
     <row r="130" spans="1:14">
       <c r="A130" s="57" t="s">
-        <v>503</v>
+        <v>489</v>
       </c>
       <c r="B130">
         <v>304</v>
@@ -5939,7 +5781,7 @@
         <v>1</v>
       </c>
       <c r="E130" s="15" t="s">
-        <v>519</v>
+        <v>505</v>
       </c>
       <c r="F130" s="79" t="s">
         <v>280</v>
@@ -5957,12 +5799,12 @@
         <v>16</v>
       </c>
       <c r="N130" s="62" t="s">
-        <v>642</v>
+        <v>600</v>
       </c>
     </row>
     <row r="133" spans="1:14">
       <c r="G133" s="14" t="s">
-        <v>691</v>
+        <v>648</v>
       </c>
     </row>
     <row r="134" spans="1:14">
@@ -5980,7 +5822,7 @@
         <v>33</v>
       </c>
       <c r="G136" s="5" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="137" spans="1:14">
@@ -6341,7 +6183,7 @@
       </c>
       <c r="B2" s="23" t="str">
         <f>Setup!G5</f>
-        <v>VA General, Test duplicates, Non Deep South, Non-bilingual</v>
+        <v>GA Primary, CD 6 &amp; 13, BIPOC voters</v>
       </c>
       <c r="C2" s="23"/>
     </row>
@@ -6351,16 +6193,16 @@
       </c>
       <c r="D3" t="str">
         <f>Setup!$G$14</f>
-        <v>General Election 7-2023</v>
+        <v>Primary 1-2024</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="B4" s="9"/>
       <c r="C4" s="33" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>394</v>
+        <v>381</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -6369,10 +6211,10 @@
         <v>274</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>393</v>
+        <v>380</v>
       </c>
       <c r="E5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="J5" s="15"/>
     </row>
@@ -6383,10 +6225,10 @@
         <v>275</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="I6" s="26"/>
     </row>
@@ -6394,13 +6236,13 @@
       <c r="A7" s="17"/>
       <c r="B7" s="9"/>
       <c r="C7" s="33" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -6420,7 +6262,7 @@
         <v>345</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>428</v>
+        <v>415</v>
       </c>
       <c r="E9" s="22" t="s">
         <v>197</v>
@@ -6432,10 +6274,10 @@
         <v>198</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="J9" s="22" t="s">
         <v>199</v>
@@ -6450,7 +6292,7 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>395</v>
+        <v>382</v>
       </c>
       <c r="B10" s="24">
         <v>3251</v>
@@ -6477,7 +6319,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>396</v>
+        <v>383</v>
       </c>
       <c r="B11">
         <v>5017</v>
@@ -6501,7 +6343,7 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B12">
         <v>10568</v>
@@ -6525,7 +6367,7 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>397</v>
+        <v>384</v>
       </c>
       <c r="B13">
         <v>4828</v>
@@ -6549,7 +6391,7 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>398</v>
+        <v>385</v>
       </c>
       <c r="B14">
         <v>896</v>
@@ -6573,7 +6415,7 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>399</v>
+        <v>386</v>
       </c>
       <c r="B15">
         <v>707</v>
@@ -6597,7 +6439,7 @@
     </row>
     <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>400</v>
+        <v>387</v>
       </c>
       <c r="B16">
         <v>1965</v>
@@ -6621,7 +6463,7 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>401</v>
+        <v>388</v>
       </c>
       <c r="B17">
         <v>799</v>
@@ -6645,7 +6487,7 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>402</v>
+        <v>389</v>
       </c>
       <c r="B18">
         <v>1191</v>
@@ -6669,7 +6511,7 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>403</v>
+        <v>390</v>
       </c>
       <c r="B19">
         <v>949</v>
@@ -6693,7 +6535,7 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>404</v>
+        <v>391</v>
       </c>
       <c r="B20">
         <v>10417</v>
@@ -6717,7 +6559,7 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>405</v>
+        <v>392</v>
       </c>
       <c r="B21">
         <v>17074</v>
@@ -6741,7 +6583,7 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>406</v>
+        <v>393</v>
       </c>
       <c r="B22">
         <v>3692</v>
@@ -6765,7 +6607,7 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>407</v>
+        <v>394</v>
       </c>
       <c r="B23">
         <v>514</v>
@@ -6789,7 +6631,7 @@
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>408</v>
+        <v>395</v>
       </c>
       <c r="B24">
         <v>417</v>
@@ -6813,7 +6655,7 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
       <c r="B25">
         <v>2252</v>
@@ -6837,7 +6679,7 @@
     </row>
     <row r="26" spans="1:9">
       <c r="A26" t="s">
-        <v>410</v>
+        <v>397</v>
       </c>
       <c r="B26">
         <v>1393</v>
@@ -6861,7 +6703,7 @@
     </row>
     <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>411</v>
+        <v>398</v>
       </c>
       <c r="B27">
         <v>1535</v>
@@ -6885,7 +6727,7 @@
     </row>
     <row r="28" spans="1:9">
       <c r="A28" t="s">
-        <v>412</v>
+        <v>399</v>
       </c>
       <c r="B28">
         <v>4348</v>
@@ -6909,7 +6751,7 @@
     </row>
     <row r="29" spans="1:9">
       <c r="A29" t="s">
-        <v>413</v>
+        <v>400</v>
       </c>
       <c r="B29">
         <v>3768</v>
@@ -6933,7 +6775,7 @@
     </row>
     <row r="30" spans="1:9">
       <c r="A30" t="s">
-        <v>414</v>
+        <v>401</v>
       </c>
       <c r="B30">
         <v>1255</v>
@@ -6957,7 +6799,7 @@
     </row>
     <row r="31" spans="1:9">
       <c r="A31" t="s">
-        <v>415</v>
+        <v>402</v>
       </c>
       <c r="B31">
         <v>894</v>
@@ -6981,7 +6823,7 @@
     </row>
     <row r="32" spans="1:9">
       <c r="A32" t="s">
-        <v>416</v>
+        <v>403</v>
       </c>
       <c r="B32">
         <v>22515</v>
@@ -7005,7 +6847,7 @@
     </row>
     <row r="33" spans="1:9">
       <c r="A33" t="s">
-        <v>417</v>
+        <v>404</v>
       </c>
       <c r="B33">
         <v>1581</v>
@@ -7029,7 +6871,7 @@
     </row>
     <row r="34" spans="1:9">
       <c r="A34" t="s">
-        <v>418</v>
+        <v>405</v>
       </c>
       <c r="B34">
         <v>52</v>
@@ -7053,7 +6895,7 @@
     </row>
     <row r="35" spans="1:9">
       <c r="A35" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B35">
         <v>4511</v>
@@ -7077,7 +6919,7 @@
     </row>
     <row r="36" spans="1:9">
       <c r="A36" t="s">
-        <v>419</v>
+        <v>406</v>
       </c>
       <c r="B36">
         <v>14433</v>
@@ -7101,7 +6943,7 @@
     </row>
     <row r="37" spans="1:9">
       <c r="A37" t="s">
-        <v>420</v>
+        <v>407</v>
       </c>
       <c r="B37">
         <v>1226</v>
@@ -7125,7 +6967,7 @@
     </row>
     <row r="38" spans="1:9">
       <c r="A38" t="s">
-        <v>421</v>
+        <v>408</v>
       </c>
       <c r="B38">
         <v>2925</v>
@@ -7149,7 +6991,7 @@
     </row>
     <row r="39" spans="1:9">
       <c r="A39" t="s">
-        <v>422</v>
+        <v>409</v>
       </c>
       <c r="B39">
         <v>11828</v>
@@ -7173,7 +7015,7 @@
     </row>
     <row r="40" spans="1:9">
       <c r="A40" t="s">
-        <v>423</v>
+        <v>410</v>
       </c>
       <c r="B40">
         <v>13379</v>
@@ -7197,7 +7039,7 @@
     </row>
     <row r="41" spans="1:9">
       <c r="A41" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="B41">
         <v>13660</v>
@@ -7221,7 +7063,7 @@
     </row>
     <row r="42" spans="1:9">
       <c r="A42" t="s">
-        <v>424</v>
+        <v>411</v>
       </c>
       <c r="B42">
         <v>37065</v>
@@ -7246,7 +7088,7 @@
     </row>
     <row r="43" spans="1:9">
       <c r="A43" t="s">
-        <v>425</v>
+        <v>412</v>
       </c>
       <c r="B43">
         <v>2767</v>
@@ -7270,7 +7112,7 @@
     </row>
     <row r="44" spans="1:9">
       <c r="A44" t="s">
-        <v>426</v>
+        <v>413</v>
       </c>
       <c r="B44">
         <v>964</v>
@@ -7294,7 +7136,7 @@
     </row>
     <row r="45" spans="1:9">
       <c r="A45" t="s">
-        <v>427</v>
+        <v>414</v>
       </c>
       <c r="B45">
         <v>4470</v>
@@ -10530,21 +10372,24 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>718</v>
+        <v>668</v>
       </c>
       <c r="B1" s="4" t="b">
         <v>1</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>720</v>
+        <v>670</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>719</v>
+        <v>669</v>
       </c>
       <c r="B2" s="4">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>688</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="17">
@@ -10564,16 +10409,16 @@
         <v>189</v>
       </c>
       <c r="F3" s="51" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>542</v>
+        <v>527</v>
       </c>
       <c r="H3" s="52" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="53" t="s">
-        <v>556</v>
+        <v>530</v>
       </c>
       <c r="K3" s="14"/>
       <c r="L3" s="14"/>
@@ -10581,16 +10426,22 @@
     </row>
     <row r="4" spans="1:13" ht="15">
       <c r="A4" t="s">
-        <v>559</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>544</v>
+        <v>674</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="4">
+        <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>388</v>
+        <v>675</v>
       </c>
       <c r="J4" s="53" t="s">
-        <v>574</v>
+        <v>533</v>
       </c>
       <c r="K4" s="14"/>
       <c r="L4" s="14"/>
@@ -10598,277 +10449,86 @@
     </row>
     <row r="5" spans="1:13" ht="15">
       <c r="A5" t="s">
-        <v>560</v>
+        <v>676</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>1</v>
       </c>
       <c r="F5" s="4">
-        <v>4</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>545</v>
+        <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>388</v>
+        <v>675</v>
       </c>
       <c r="J5" s="53" t="s">
-        <v>557</v>
+        <v>531</v>
       </c>
       <c r="K5" s="14"/>
       <c r="L5" s="14"/>
       <c r="M5" s="14"/>
     </row>
     <row r="6" spans="1:13" ht="15">
-      <c r="A6" t="s">
-        <v>561</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F6" s="4">
-        <v>3</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>546</v>
-      </c>
-      <c r="H6" t="s">
-        <v>573</v>
-      </c>
+      <c r="H6"/>
       <c r="J6" s="53" t="s">
-        <v>558</v>
+        <v>532</v>
       </c>
       <c r="K6" s="14"/>
       <c r="L6" s="14"/>
       <c r="M6" s="14"/>
     </row>
     <row r="7" spans="1:13" ht="15">
-      <c r="A7" t="s">
-        <v>383</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F7" s="4">
-        <v>3</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>547</v>
-      </c>
-      <c r="H7" t="s">
-        <v>388</v>
-      </c>
+      <c r="H7"/>
     </row>
     <row r="8" spans="1:13" ht="15">
-      <c r="A8" t="s">
-        <v>384</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F8" s="4">
-        <v>3</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>548</v>
-      </c>
-      <c r="H8" t="s">
-        <v>388</v>
-      </c>
+      <c r="H8"/>
       <c r="J8" s="53" t="s">
-        <v>575</v>
+        <v>534</v>
       </c>
       <c r="K8" s="14"/>
       <c r="L8" s="14"/>
       <c r="M8" s="14"/>
     </row>
     <row r="9" spans="1:13" ht="15">
-      <c r="A9" t="s">
-        <v>562</v>
-      </c>
-      <c r="F9" s="4">
-        <v>5</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>549</v>
-      </c>
-      <c r="H9" t="s">
-        <v>388</v>
-      </c>
+      <c r="H9"/>
     </row>
     <row r="10" spans="1:13" ht="15">
-      <c r="A10" t="s">
-        <v>385</v>
-      </c>
-      <c r="F10" s="4">
-        <v>4</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>550</v>
-      </c>
-      <c r="H10" t="s">
-        <v>388</v>
-      </c>
+      <c r="H10"/>
     </row>
     <row r="11" spans="1:13" ht="15">
-      <c r="A11" t="s">
-        <v>563</v>
-      </c>
-      <c r="F11" s="4">
-        <v>3</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>544</v>
-      </c>
-      <c r="H11" t="s">
-        <v>573</v>
-      </c>
+      <c r="H11"/>
     </row>
     <row r="12" spans="1:13" ht="15">
-      <c r="A12" t="s">
-        <v>564</v>
-      </c>
-      <c r="F12" s="4">
-        <v>2</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>545</v>
-      </c>
-      <c r="H12" t="s">
-        <v>573</v>
-      </c>
+      <c r="H12"/>
     </row>
     <row r="13" spans="1:13" ht="15">
-      <c r="A13" t="s">
-        <v>565</v>
-      </c>
-      <c r="F13" s="4">
-        <v>1</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>546</v>
-      </c>
-      <c r="H13" t="s">
-        <v>573</v>
-      </c>
+      <c r="H13"/>
     </row>
     <row r="14" spans="1:13" ht="15">
-      <c r="A14" t="s">
-        <v>566</v>
-      </c>
-      <c r="F14" s="4">
-        <v>5</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>547</v>
-      </c>
-      <c r="H14" t="s">
-        <v>573</v>
-      </c>
+      <c r="H14"/>
     </row>
     <row r="15" spans="1:13" ht="15">
-      <c r="A15" t="s">
-        <v>567</v>
-      </c>
-      <c r="F15" s="4">
-        <v>4</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>548</v>
-      </c>
-      <c r="H15" t="s">
-        <v>573</v>
-      </c>
+      <c r="H15"/>
     </row>
     <row r="16" spans="1:13" ht="15">
-      <c r="A16" t="s">
-        <v>568</v>
-      </c>
-      <c r="F16" s="4">
-        <v>3</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>549</v>
-      </c>
-      <c r="H16" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="15">
-      <c r="A17" t="s">
-        <v>569</v>
-      </c>
-      <c r="F17" s="4">
-        <v>2</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>550</v>
-      </c>
-      <c r="H17" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="15">
-      <c r="A18" t="s">
-        <v>570</v>
-      </c>
-      <c r="F18" s="4">
-        <v>1</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>544</v>
-      </c>
-      <c r="H18" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="15">
-      <c r="A19" t="s">
-        <v>571</v>
-      </c>
-      <c r="F19" s="4">
-        <v>1</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>545</v>
-      </c>
-      <c r="H19" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="15">
-      <c r="A20" t="s">
-        <v>374</v>
-      </c>
-      <c r="F20" s="4">
-        <v>1</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>546</v>
-      </c>
-      <c r="H20" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="15">
-      <c r="A21" t="s">
-        <v>572</v>
-      </c>
-      <c r="F21" s="4">
-        <v>1</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>547</v>
-      </c>
-      <c r="H21" t="s">
-        <v>387</v>
-      </c>
+      <c r="H16"/>
+    </row>
+    <row r="17" spans="8:8" ht="15">
+      <c r="H17"/>
+    </row>
+    <row r="18" spans="8:8" ht="15">
+      <c r="H18"/>
+    </row>
+    <row r="19" spans="8:8" ht="15">
+      <c r="H19"/>
+    </row>
+    <row r="20" spans="8:8" ht="15">
+      <c r="H20"/>
+    </row>
+    <row r="21" spans="8:8" ht="15">
+      <c r="H21"/>
     </row>
   </sheetData>
   <sortState ref="A4:E7">
@@ -10891,7 +10551,7 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="54" t="s">
-        <v>577</v>
+        <v>536</v>
       </c>
       <c r="K1" t="s">
         <v>273</v>
@@ -10909,7 +10569,7 @@
     </row>
     <row r="5" spans="1:15">
       <c r="M5" s="53" t="s">
-        <v>692</v>
+        <v>649</v>
       </c>
       <c r="N5" s="14"/>
       <c r="O5" s="14"/>
@@ -10919,7 +10579,7 @@
         <v>322</v>
       </c>
       <c r="M6" s="53" t="s">
-        <v>694</v>
+        <v>651</v>
       </c>
       <c r="N6" s="14"/>
       <c r="O6" s="14"/>
@@ -10950,7 +10610,7 @@
       </c>
       <c r="C12" s="15"/>
       <c r="M12" s="53" t="s">
-        <v>693</v>
+        <v>650</v>
       </c>
       <c r="N12" s="14"/>
       <c r="O12" s="14"/>
@@ -11011,7 +10671,7 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="54" t="s">
-        <v>576</v>
+        <v>535</v>
       </c>
       <c r="L1" t="s">
         <v>273</v>
@@ -11031,10 +10691,10 @@
     <row r="4" spans="1:15">
       <c r="A4" s="54"/>
       <c r="B4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="L4" s="53" t="s">
-        <v>692</v>
+        <v>649</v>
       </c>
       <c r="M4" s="14"/>
       <c r="N4" s="14"/>
@@ -11042,7 +10702,7 @@
     <row r="5" spans="1:15">
       <c r="A5" s="54"/>
       <c r="L5" s="53" t="s">
-        <v>694</v>
+        <v>651</v>
       </c>
       <c r="M5" s="14"/>
       <c r="N5" s="14"/>
@@ -11059,7 +10719,7 @@
         <v>246</v>
       </c>
       <c r="L7" s="53" t="s">
-        <v>695</v>
+        <v>652</v>
       </c>
       <c r="M7" s="14"/>
       <c r="N7" s="14"/>
@@ -11082,10 +10742,10 @@
     <row r="10" spans="1:15">
       <c r="A10" s="54"/>
       <c r="C10" t="s">
-        <v>578</v>
+        <v>537</v>
       </c>
       <c r="L10" s="53" t="s">
-        <v>696</v>
+        <v>653</v>
       </c>
       <c r="M10" s="14"/>
       <c r="N10" s="14"/>
@@ -11174,7 +10834,7 @@
     <row r="23" spans="1:13">
       <c r="A23" s="54"/>
       <c r="B23" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="M23" s="55"/>
     </row>
@@ -11188,49 +10848,49 @@
     <row r="25" spans="1:13">
       <c r="A25" s="54"/>
       <c r="C25" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="M25" s="55"/>
     </row>
     <row r="26" spans="1:13">
       <c r="A26" s="54"/>
       <c r="D26" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="M26" s="55"/>
     </row>
     <row r="27" spans="1:13">
       <c r="A27" s="54"/>
       <c r="C27" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="M27" s="55"/>
     </row>
     <row r="28" spans="1:13">
       <c r="A28" s="54"/>
       <c r="D28" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M28" s="55"/>
     </row>
     <row r="29" spans="1:13">
       <c r="A29" s="54"/>
       <c r="C29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="M29" s="55"/>
     </row>
     <row r="30" spans="1:13">
       <c r="A30" s="54"/>
       <c r="D30" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="M30" s="55"/>
     </row>
     <row r="31" spans="1:13">
       <c r="A31" s="54"/>
       <c r="C31" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="M31" s="55"/>
     </row>
@@ -11245,7 +10905,7 @@
     </row>
     <row r="36" spans="2:2">
       <c r="B36" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="38" spans="2:2">
@@ -11255,7 +10915,7 @@
     </row>
     <row r="39" spans="2:2">
       <c r="B39" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="41" spans="2:2">
@@ -11280,22 +10940,22 @@
     </row>
     <row r="47" spans="2:2">
       <c r="B47" t="s">
-        <v>553</v>
+        <v>529</v>
       </c>
     </row>
     <row r="48" spans="2:2">
       <c r="B48" t="s">
-        <v>551</v>
+        <v>683</v>
       </c>
     </row>
     <row r="50" spans="2:2">
       <c r="B50" t="s">
-        <v>552</v>
+        <v>528</v>
       </c>
     </row>
     <row r="51" spans="2:2">
       <c r="B51" t="s">
-        <v>555</v>
+        <v>684</v>
       </c>
     </row>
     <row r="54" spans="2:2">
@@ -11310,47 +10970,47 @@
     </row>
     <row r="56" spans="2:2">
       <c r="B56" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="59" spans="2:2">
       <c r="B59" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="60" spans="2:2">
       <c r="B60" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="62" spans="2:2">
       <c r="B62" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="63" spans="2:2">
       <c r="B63" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="66" spans="2:2">
       <c r="B66" t="s">
-        <v>708</v>
+        <v>663</v>
       </c>
     </row>
     <row r="67" spans="2:2">
       <c r="B67" t="s">
-        <v>710</v>
+        <v>682</v>
       </c>
     </row>
     <row r="68" spans="2:2">
       <c r="B68" t="s">
-        <v>713</v>
+        <v>681</v>
       </c>
     </row>
     <row r="69" spans="2:2">
       <c r="B69" t="s">
-        <v>723</v>
+        <v>673</v>
       </c>
     </row>
   </sheetData>
@@ -11381,7 +11041,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="B4" t="s">
-        <v>459</v>
+        <v>445</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -11391,7 +11051,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="I6" s="53" t="s">
-        <v>692</v>
+        <v>649</v>
       </c>
       <c r="J6" s="14"/>
       <c r="K6" s="14"/>
@@ -11401,14 +11061,14 @@
         <v>292</v>
       </c>
       <c r="I7" s="53" t="s">
-        <v>694</v>
+        <v>651</v>
       </c>
       <c r="J7" s="14"/>
       <c r="K7" s="14"/>
     </row>
     <row r="8" spans="1:12">
       <c r="I8" s="53" t="s">
-        <v>697</v>
+        <v>654</v>
       </c>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -11423,7 +11083,7 @@
         <v>294</v>
       </c>
       <c r="I10" s="53" t="s">
-        <v>698</v>
+        <v>655</v>
       </c>
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
@@ -11433,7 +11093,7 @@
         <v>295</v>
       </c>
       <c r="I11" s="53" t="s">
-        <v>699</v>
+        <v>656</v>
       </c>
       <c r="J11" s="14"/>
       <c r="K11" s="14"/>
@@ -11441,7 +11101,7 @@
     </row>
     <row r="12" spans="1:12">
       <c r="I12" s="53" t="s">
-        <v>700</v>
+        <v>657</v>
       </c>
       <c r="J12" s="14"/>
       <c r="K12" s="14"/>
@@ -11616,27 +11276,22 @@
     </row>
     <row r="64" spans="2:3">
       <c r="B64" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="65" spans="2:8">
-      <c r="B65" t="s">
-        <v>380</v>
+        <v>687</v>
       </c>
     </row>
     <row r="67" spans="2:8">
       <c r="B67" t="s">
-        <v>540</v>
+        <v>525</v>
       </c>
     </row>
     <row r="68" spans="2:8">
       <c r="B68" t="s">
-        <v>722</v>
+        <v>672</v>
       </c>
     </row>
     <row r="69" spans="2:8">
       <c r="B69" s="14" t="s">
-        <v>721</v>
+        <v>671</v>
       </c>
       <c r="C69" s="14"/>
       <c r="D69" s="14"/>
@@ -11688,7 +11343,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="B4">
         <v>23321</v>
@@ -11765,12 +11420,12 @@
   <sheetData>
     <row r="1" spans="1:3" ht="26">
       <c r="A1" s="46" t="s">
-        <v>435</v>
+        <v>422</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18">
       <c r="B3" s="47" t="s">
-        <v>429</v>
+        <v>416</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="18">
@@ -11779,18 +11434,18 @@
     <row r="5" spans="1:3" ht="18">
       <c r="A5" s="44"/>
       <c r="B5" s="45" t="s">
-        <v>449</v>
+        <v>436</v>
       </c>
       <c r="C5" t="s">
-        <v>430</v>
+        <v>417</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="B6" s="17" t="s">
-        <v>446</v>
+        <v>433</v>
       </c>
       <c r="C6" s="48" t="s">
-        <v>451</v>
+        <v>438</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -11805,15 +11460,15 @@
     </row>
     <row r="10" spans="1:3" ht="32">
       <c r="B10" s="45" t="s">
-        <v>436</v>
+        <v>423</v>
       </c>
       <c r="C10" s="48" t="s">
-        <v>434</v>
+        <v>421</v>
       </c>
     </row>
     <row r="12" spans="1:3" hidden="1" outlineLevel="1">
       <c r="B12" t="s">
-        <v>431</v>
+        <v>418</v>
       </c>
       <c r="C12" s="26">
         <f>SEARCH($C$10,$C$6)</f>
@@ -11822,7 +11477,7 @@
     </row>
     <row r="13" spans="1:3" hidden="1" outlineLevel="1">
       <c r="B13" t="s">
-        <v>432</v>
+        <v>419</v>
       </c>
       <c r="C13" t="str">
         <f>"**/" &amp; RIGHT($C$6,LEN($C$6)-$C$12+1)</f>
@@ -11831,7 +11486,7 @@
     </row>
     <row r="14" spans="1:3" hidden="1" outlineLevel="1">
       <c r="B14" t="s">
-        <v>433</v>
+        <v>420</v>
       </c>
       <c r="C14" t="str">
         <f>RIGHT($C$13,LEN($C$13)-FIND("|",SUBSTITUTE($C$13,"-","|",
@@ -11842,7 +11497,7 @@
     <row r="15" spans="1:3" collapsed="1"/>
     <row r="16" spans="1:3">
       <c r="B16" s="17" t="s">
-        <v>441</v>
+        <v>428</v>
       </c>
       <c r="C16" s="49" t="str">
         <f>LEFT($C$13,LEN($C$13)-LEN($C$14)) &amp; "[filename]/*.pdf"</f>
@@ -11851,15 +11506,15 @@
     </row>
     <row r="17" spans="2:3">
       <c r="B17" s="17" t="s">
-        <v>447</v>
+        <v>434</v>
       </c>
       <c r="C17" t="s">
-        <v>445</v>
+        <v>432</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="18">
       <c r="B21" s="47" t="s">
-        <v>437</v>
+        <v>424</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="18">
@@ -11867,26 +11522,26 @@
     </row>
     <row r="23" spans="2:3">
       <c r="B23" s="17" t="s">
-        <v>450</v>
+        <v>437</v>
       </c>
       <c r="C23" t="s">
-        <v>438</v>
+        <v>425</v>
       </c>
     </row>
     <row r="24" spans="2:3">
       <c r="B24" s="17" t="s">
-        <v>448</v>
+        <v>435</v>
       </c>
       <c r="C24" s="48" t="s">
-        <v>452</v>
+        <v>439</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="32">
       <c r="B27" s="45" t="s">
-        <v>439</v>
+        <v>426</v>
       </c>
       <c r="C27" s="48" t="s">
-        <v>434</v>
+        <v>421</v>
       </c>
     </row>
     <row r="29" spans="2:3">
@@ -11897,10 +11552,10 @@
     </row>
     <row r="30" spans="2:3" ht="32">
       <c r="B30" s="45" t="s">
-        <v>443</v>
+        <v>430</v>
       </c>
       <c r="C30" s="48" t="s">
-        <v>453</v>
+        <v>440</v>
       </c>
     </row>
     <row r="31" spans="2:3">
@@ -11912,7 +11567,7 @@
     <row r="33" spans="2:3" hidden="1" outlineLevel="1"/>
     <row r="34" spans="2:3" hidden="1" outlineLevel="1">
       <c r="B34" t="s">
-        <v>431</v>
+        <v>418</v>
       </c>
       <c r="C34" s="26">
         <f>SEARCH($C$27,$C$24)</f>
@@ -11921,7 +11576,7 @@
     </row>
     <row r="35" spans="2:3" hidden="1" outlineLevel="1">
       <c r="B35" t="s">
-        <v>432</v>
+        <v>419</v>
       </c>
       <c r="C35" t="str">
         <f>"**/" &amp; RIGHT($C$24,LEN($C$24)-$C$34+1)</f>
@@ -11930,7 +11585,7 @@
     </row>
     <row r="36" spans="2:3" hidden="1" outlineLevel="1">
       <c r="B36" t="s">
-        <v>440</v>
+        <v>427</v>
       </c>
       <c r="C36" t="str">
         <f>SUBSTITUTE($C$35,$C$30,"[filename]",1)</f>
@@ -11941,7 +11596,7 @@
     <row r="38" spans="2:3" collapsed="1"/>
     <row r="39" spans="2:3">
       <c r="B39" s="17" t="s">
-        <v>442</v>
+        <v>429</v>
       </c>
       <c r="C39" s="49" t="str">
         <f>SUBSTITUTE($C$36,".csv","[filecounter].csv",1)</f>
@@ -11950,10 +11605,10 @@
     </row>
     <row r="40" spans="2:3">
       <c r="B40" s="17" t="s">
-        <v>447</v>
+        <v>434</v>
       </c>
       <c r="C40" t="s">
-        <v>444</v>
+        <v>431</v>
       </c>
     </row>
   </sheetData>
@@ -11995,7 +11650,7 @@
       </c>
       <c r="B2" s="23" t="str">
         <f>Setup!G5</f>
-        <v>VA General, Test duplicates, Non Deep South, Non-bilingual</v>
+        <v>GA Primary, CD 6 &amp; 13, BIPOC voters</v>
       </c>
       <c r="C2" s="23"/>
     </row>
@@ -12005,16 +11660,16 @@
       </c>
       <c r="D3" t="str">
         <f>Setup!$G$14</f>
-        <v>General Election 7-2023</v>
+        <v>Primary 1-2024</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="B4" s="9"/>
       <c r="C4" s="33" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>394</v>
+        <v>381</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -12023,10 +11678,10 @@
         <v>274</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>393</v>
+        <v>380</v>
       </c>
       <c r="E5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="J5" s="15"/>
     </row>
@@ -12037,10 +11692,10 @@
         <v>275</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="I6" s="26"/>
     </row>
@@ -12048,13 +11703,13 @@
       <c r="A7" s="17"/>
       <c r="B7" s="9"/>
       <c r="C7" s="33" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -12074,7 +11729,7 @@
         <v>345</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>428</v>
+        <v>415</v>
       </c>
       <c r="E9" s="22" t="s">
         <v>197</v>
@@ -12086,10 +11741,10 @@
         <v>198</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="J9" s="22" t="s">
         <v>199</v>
@@ -12104,7 +11759,7 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>395</v>
+        <v>382</v>
       </c>
       <c r="B10" s="24">
         <v>29</v>
@@ -12131,7 +11786,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B11">
         <v>6799</v>
@@ -12155,7 +11810,7 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>397</v>
+        <v>384</v>
       </c>
       <c r="B12">
         <v>10678</v>
@@ -12179,7 +11834,7 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>455</v>
+        <v>441</v>
       </c>
       <c r="B13">
         <v>1208</v>
@@ -12203,7 +11858,7 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>398</v>
+        <v>385</v>
       </c>
       <c r="B14">
         <v>187</v>
@@ -12227,7 +11882,7 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>399</v>
+        <v>386</v>
       </c>
       <c r="B15">
         <v>35</v>
@@ -12251,7 +11906,7 @@
     </row>
     <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>456</v>
+        <v>442</v>
       </c>
       <c r="B16">
         <v>6876</v>
@@ -12275,7 +11930,7 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>403</v>
+        <v>390</v>
       </c>
       <c r="B17">
         <v>12</v>
@@ -12299,7 +11954,7 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>406</v>
+        <v>393</v>
       </c>
       <c r="B18">
         <v>117</v>
@@ -12323,7 +11978,7 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>407</v>
+        <v>394</v>
       </c>
       <c r="B19">
         <v>4277</v>
@@ -12347,7 +12002,7 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>457</v>
+        <v>443</v>
       </c>
       <c r="B20">
         <v>717</v>
@@ -12371,7 +12026,7 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>419</v>
+        <v>406</v>
       </c>
       <c r="B21">
         <v>16720</v>
@@ -12395,7 +12050,7 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>421</v>
+        <v>408</v>
       </c>
       <c r="B22">
         <v>10</v>
@@ -12419,7 +12074,7 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="B23">
         <v>56</v>
@@ -12443,7 +12098,7 @@
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>458</v>
+        <v>444</v>
       </c>
       <c r="B24">
         <v>889</v>
@@ -12467,7 +12122,7 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>426</v>
+        <v>413</v>
       </c>
       <c r="B25">
         <v>5</v>

</xml_diff>

<commit_message>
add setup_backward_compatability but then didn't run cause pull_group vars in filelist, not standard format
</commit_message>
<xml_diff>
--- a/WorkCampaign/ROVCleaver UniversalSetup.xlsx
+++ b/WorkCampaign/ROVCleaver UniversalSetup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/TestInputFiles/TestCampaigns/Test GA Primary 1-2024/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/Postcard Files/PythonPrograms/Development/ROVCleaver/WorkCampaign/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0759BA38-6B68-2F46-85A5-22203A62A4AF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D235DFA-B0B5-B14A-9DB1-285A20E00D69}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3800" yWindow="2940" windowWidth="25940" windowHeight="14100" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
+    <workbookView xWindow="2860" yWindow="2940" windowWidth="25940" windowHeight="14100" activeTab="1" xr2:uid="{A3D11580-81DE-480D-BED2-9222F9450ACB}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="39" r:id="rId1"/>
@@ -126,6 +126,82 @@
     <author>Brian Kramer</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{7AC06AEF-0766-3348-9105-2C1D6CC0B050}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Brian Kramer:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Do not change this text as it is used in the program to verify the file format.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{67AFEAC4-95D5-7049-8802-A61353A9A5CE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Brian Kramer:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Do not change this text as it is used in the program to verify the file format.</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="A3" authorId="0" shapeId="0" xr:uid="{FE08C722-80B9-E64F-960D-B18EDD4A84CB}">
       <text>
         <r>
@@ -146,7 +222,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Copy file names from RawData.  In Finder, select all files (Ctrl + A) &gt; right click &gt; copy</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Copy file names from RawData.  In Finder, select all files (Ctrl + A) &gt; right click &gt; copy</t>
         </r>
       </text>
     </comment>
@@ -2658,7 +2743,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(\ #,##0_);_(\ \(#,##0\);_(&quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="44">
+  <fonts count="45">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2968,6 +3053,12 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>

</xml_diff>